<commit_message>
Update ArcMap palette with corrections analysis and enhanced reference assets
</commit_message>
<xml_diff>
--- a/color-palettes/arcmap-standard-palette/ArcMap_Color_Palette.xlsx
+++ b/color-palettes/arcmap-standard-palette/ArcMap_Color_Palette.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Palette Grid'!$A$1:$L$43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Color Reference'!$A$1:$J$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Color Reference'!$A$1:$M$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -5340,7 +5340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J121"/>
+  <dimension ref="A1:M121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5351,8 +5351,11 @@
     <col width="6" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="52" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -5398,10 +5401,25 @@
       </c>
       <c r="I1" s="483" t="inlineStr">
         <is>
+          <t>H°</t>
+        </is>
+      </c>
+      <c r="J1" s="483" t="inlineStr">
+        <is>
+          <t>S%</t>
+        </is>
+      </c>
+      <c r="K1" s="483" t="inlineStr">
+        <is>
+          <t>V%</t>
+        </is>
+      </c>
+      <c r="L1" s="483" t="inlineStr">
+        <is>
           <t>Swatch</t>
         </is>
       </c>
-      <c r="J1" s="483" t="inlineStr">
+      <c r="M1" s="483" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -5436,8 +5454,17 @@
           <t>#FFFFFF</t>
         </is>
       </c>
-      <c r="I2" s="487" t="inlineStr"/>
-      <c r="J2" s="488" t="inlineStr">
+      <c r="I2" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L2" s="487" t="inlineStr"/>
+      <c r="M2" s="488" t="inlineStr">
         <is>
           <t>Pure white; blank paper, unmapped areas</t>
         </is>
@@ -5472,8 +5499,17 @@
           <t>#FFBEBE</t>
         </is>
       </c>
-      <c r="I3" s="489" t="inlineStr"/>
-      <c r="J3" s="488" t="inlineStr">
+      <c r="I3" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="484" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="K3" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L3" s="489" t="inlineStr"/>
+      <c r="M3" s="488" t="inlineStr">
         <is>
           <t>Pale warm pink; soft residential fills</t>
         </is>
@@ -5508,8 +5544,17 @@
           <t>#FFEBBE</t>
         </is>
       </c>
-      <c r="I4" s="490" t="inlineStr"/>
-      <c r="J4" s="488" t="inlineStr">
+      <c r="I4" s="484" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="J4" s="484" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="K4" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L4" s="490" t="inlineStr"/>
+      <c r="M4" s="488" t="inlineStr">
         <is>
           <t>Pale warm tan; dry land, sand</t>
         </is>
@@ -5544,8 +5589,17 @@
           <t>#FFEBAF</t>
         </is>
       </c>
-      <c r="I5" s="491" t="inlineStr"/>
-      <c r="J5" s="488" t="inlineStr">
+      <c r="I5" s="484" t="n">
+        <v>45</v>
+      </c>
+      <c r="J5" s="484" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="K5" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L5" s="491" t="inlineStr"/>
+      <c r="M5" s="488" t="inlineStr">
         <is>
           <t>Pale golden beige; wheat fields, prairie</t>
         </is>
@@ -5580,8 +5634,17 @@
           <t>#FFFFBE</t>
         </is>
       </c>
-      <c r="I6" s="492" t="inlineStr"/>
-      <c r="J6" s="488" t="inlineStr">
+      <c r="I6" s="484" t="n">
+        <v>60</v>
+      </c>
+      <c r="J6" s="484" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="K6" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L6" s="492" t="inlineStr"/>
+      <c r="M6" s="488" t="inlineStr">
         <is>
           <t>Pale warm yellow; light agricultural zones</t>
         </is>
@@ -5616,8 +5679,17 @@
           <t>#E9FFBE</t>
         </is>
       </c>
-      <c r="I7" s="493" t="inlineStr"/>
-      <c r="J7" s="488" t="inlineStr">
+      <c r="I7" s="484" t="n">
+        <v>80.3</v>
+      </c>
+      <c r="J7" s="484" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="K7" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L7" s="493" t="inlineStr"/>
+      <c r="M7" s="488" t="inlineStr">
         <is>
           <t>Pale yellow-green; light vegetation, meadows</t>
         </is>
@@ -5652,8 +5724,17 @@
           <t>#D3FFBE</t>
         </is>
       </c>
-      <c r="I8" s="494" t="inlineStr"/>
-      <c r="J8" s="488" t="inlineStr">
+      <c r="I8" s="484" t="n">
+        <v>100.6</v>
+      </c>
+      <c r="J8" s="484" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="K8" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L8" s="494" t="inlineStr"/>
+      <c r="M8" s="488" t="inlineStr">
         <is>
           <t>Pale mint green; soft parks, greenspace</t>
         </is>
@@ -5688,8 +5769,17 @@
           <t>#BEFFE8</t>
         </is>
       </c>
-      <c r="I9" s="495" t="inlineStr"/>
-      <c r="J9" s="488" t="inlineStr">
+      <c r="I9" s="484" t="n">
+        <v>158.8</v>
+      </c>
+      <c r="J9" s="484" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="K9" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L9" s="495" t="inlineStr"/>
+      <c r="M9" s="488" t="inlineStr">
         <is>
           <t>Pale cool seafoam; shallow water, wetlands</t>
         </is>
@@ -5724,8 +5814,17 @@
           <t>#BEE8FF</t>
         </is>
       </c>
-      <c r="I10" s="496" t="inlineStr"/>
-      <c r="J10" s="488" t="inlineStr">
+      <c r="I10" s="484" t="n">
+        <v>201.2</v>
+      </c>
+      <c r="J10" s="484" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="K10" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L10" s="496" t="inlineStr"/>
+      <c r="M10" s="488" t="inlineStr">
         <is>
           <t>Pale cool sky; soft water fills</t>
         </is>
@@ -5760,8 +5859,17 @@
           <t>#BED2FF</t>
         </is>
       </c>
-      <c r="I11" s="497" t="inlineStr"/>
-      <c r="J11" s="488" t="inlineStr">
+      <c r="I11" s="484" t="n">
+        <v>221.5</v>
+      </c>
+      <c r="J11" s="484" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="K11" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L11" s="497" t="inlineStr"/>
+      <c r="M11" s="488" t="inlineStr">
         <is>
           <t>Pale cool periwinkle; atmospheric backgrounds</t>
         </is>
@@ -5796,8 +5904,17 @@
           <t>#E8BEFF</t>
         </is>
       </c>
-      <c r="I12" s="498" t="inlineStr"/>
-      <c r="J12" s="488" t="inlineStr">
+      <c r="I12" s="484" t="n">
+        <v>278.8</v>
+      </c>
+      <c r="J12" s="484" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="K12" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L12" s="498" t="inlineStr"/>
+      <c r="M12" s="488" t="inlineStr">
         <is>
           <t>Pale cool lavender; soft zoning overlays</t>
         </is>
@@ -5832,8 +5949,17 @@
           <t>#FFBEE8</t>
         </is>
       </c>
-      <c r="I13" s="499" t="inlineStr"/>
-      <c r="J13" s="488" t="inlineStr">
+      <c r="I13" s="484" t="n">
+        <v>321.2</v>
+      </c>
+      <c r="J13" s="484" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="K13" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L13" s="499" t="inlineStr"/>
+      <c r="M13" s="488" t="inlineStr">
         <is>
           <t>Pale warm pink-magenta; light zoning fills</t>
         </is>
@@ -5868,8 +5994,17 @@
           <t>#E1E1E1</t>
         </is>
       </c>
-      <c r="I14" s="500" t="inlineStr"/>
-      <c r="J14" s="488" t="inlineStr">
+      <c r="I14" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="484" t="n">
+        <v>88.2</v>
+      </c>
+      <c r="L14" s="500" t="inlineStr"/>
+      <c r="M14" s="488" t="inlineStr">
         <is>
           <t>Very light neutral; subtle basemap fills</t>
         </is>
@@ -5904,8 +6039,17 @@
           <t>#FF7F7F</t>
         </is>
       </c>
-      <c r="I15" s="501" t="inlineStr"/>
-      <c r="J15" s="488" t="inlineStr">
+      <c r="I15" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K15" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L15" s="501" t="inlineStr"/>
+      <c r="M15" s="488" t="inlineStr">
         <is>
           <t>Medium-light warm coral; residential districts</t>
         </is>
@@ -5940,8 +6084,17 @@
           <t>#FFA77F</t>
         </is>
       </c>
-      <c r="I16" s="502" t="inlineStr"/>
-      <c r="J16" s="488" t="inlineStr">
+      <c r="I16" s="484" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="J16" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K16" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L16" s="502" t="inlineStr"/>
+      <c r="M16" s="488" t="inlineStr">
         <is>
           <t>Light warm peach; commercial zones</t>
         </is>
@@ -5976,8 +6129,17 @@
           <t>#FFD37F</t>
         </is>
       </c>
-      <c r="I17" s="503" t="inlineStr"/>
-      <c r="J17" s="488" t="inlineStr">
+      <c r="I17" s="484" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="J17" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K17" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L17" s="503" t="inlineStr"/>
+      <c r="M17" s="488" t="inlineStr">
         <is>
           <t>Light warm gold; agricultural highlights</t>
         </is>
@@ -6012,8 +6174,17 @@
           <t>#FFFF73</t>
         </is>
       </c>
-      <c r="I18" s="504" t="inlineStr"/>
-      <c r="J18" s="488" t="inlineStr">
+      <c r="I18" s="484" t="n">
+        <v>60</v>
+      </c>
+      <c r="J18" s="484" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="K18" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L18" s="504" t="inlineStr"/>
+      <c r="M18" s="488" t="inlineStr">
         <is>
           <t>Bright warm yellow; highways, caution zones</t>
         </is>
@@ -6048,8 +6219,17 @@
           <t>#D1FF73</t>
         </is>
       </c>
-      <c r="I19" s="505" t="inlineStr"/>
-      <c r="J19" s="488" t="inlineStr">
+      <c r="I19" s="484" t="n">
+        <v>79.7</v>
+      </c>
+      <c r="J19" s="484" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="K19" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L19" s="505" t="inlineStr"/>
+      <c r="M19" s="488" t="inlineStr">
         <is>
           <t>Bright yellow-green; active vegetation</t>
         </is>
@@ -6084,8 +6264,17 @@
           <t>#A3FF73</t>
         </is>
       </c>
-      <c r="I20" s="506" t="inlineStr"/>
-      <c r="J20" s="488" t="inlineStr">
+      <c r="I20" s="484" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="J20" s="484" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="K20" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L20" s="506" t="inlineStr"/>
+      <c r="M20" s="488" t="inlineStr">
         <is>
           <t>Bright spring green; healthy crops, parks</t>
         </is>
@@ -6120,8 +6309,17 @@
           <t>#73FFDF</t>
         </is>
       </c>
-      <c r="I21" s="507" t="inlineStr"/>
-      <c r="J21" s="488" t="inlineStr">
+      <c r="I21" s="484" t="n">
+        <v>166.3</v>
+      </c>
+      <c r="J21" s="484" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="K21" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L21" s="507" t="inlineStr"/>
+      <c r="M21" s="488" t="inlineStr">
         <is>
           <t>Bright cool aqua; shallow tropical water</t>
         </is>
@@ -6156,8 +6354,17 @@
           <t>#73DFFF</t>
         </is>
       </c>
-      <c r="I22" s="508" t="inlineStr"/>
-      <c r="J22" s="488" t="inlineStr">
+      <c r="I22" s="484" t="n">
+        <v>193.7</v>
+      </c>
+      <c r="J22" s="484" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="K22" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L22" s="508" t="inlineStr"/>
+      <c r="M22" s="488" t="inlineStr">
         <is>
           <t>Bright cool cyan; pool blue, recreation</t>
         </is>
@@ -6192,8 +6399,17 @@
           <t>#73B2FF</t>
         </is>
       </c>
-      <c r="I23" s="509" t="inlineStr"/>
-      <c r="J23" s="488" t="inlineStr">
+      <c r="I23" s="484" t="n">
+        <v>213</v>
+      </c>
+      <c r="J23" s="484" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="K23" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L23" s="509" t="inlineStr"/>
+      <c r="M23" s="488" t="inlineStr">
         <is>
           <t>Bright cool cornflower; lakes, reservoirs</t>
         </is>
@@ -6228,8 +6444,17 @@
           <t>#DF73FF</t>
         </is>
       </c>
-      <c r="I24" s="510" t="inlineStr"/>
-      <c r="J24" s="488" t="inlineStr">
+      <c r="I24" s="484" t="n">
+        <v>286.3</v>
+      </c>
+      <c r="J24" s="484" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="K24" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L24" s="510" t="inlineStr"/>
+      <c r="M24" s="488" t="inlineStr">
         <is>
           <t>Bright cool orchid; special districts</t>
         </is>
@@ -6264,8 +6489,17 @@
           <t>#FF73DF</t>
         </is>
       </c>
-      <c r="I25" s="511" t="inlineStr"/>
-      <c r="J25" s="488" t="inlineStr">
+      <c r="I25" s="484" t="n">
+        <v>313.7</v>
+      </c>
+      <c r="J25" s="484" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="K25" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L25" s="511" t="inlineStr"/>
+      <c r="M25" s="488" t="inlineStr">
         <is>
           <t>Bright warm hot pink; attention-getting markers</t>
         </is>
@@ -6300,8 +6534,17 @@
           <t>#CCCCCC</t>
         </is>
       </c>
-      <c r="I26" s="512" t="inlineStr"/>
-      <c r="J26" s="488" t="inlineStr">
+      <c r="I26" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="484" t="n">
+        <v>80</v>
+      </c>
+      <c r="L26" s="512" t="inlineStr"/>
+      <c r="M26" s="488" t="inlineStr">
         <is>
           <t>Light neutral; background fills, UI</t>
         </is>
@@ -6336,8 +6579,17 @@
           <t>#FF0000</t>
         </is>
       </c>
-      <c r="I27" s="513" t="inlineStr"/>
-      <c r="J27" s="488" t="inlineStr">
+      <c r="I27" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K27" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L27" s="513" t="inlineStr"/>
+      <c r="M27" s="488" t="inlineStr">
         <is>
           <t>Pure saturated red; alerts, hazards</t>
         </is>
@@ -6372,8 +6624,17 @@
           <t>#FF5500</t>
         </is>
       </c>
-      <c r="I28" s="514" t="inlineStr"/>
-      <c r="J28" s="488" t="inlineStr">
+      <c r="I28" s="484" t="n">
+        <v>20</v>
+      </c>
+      <c r="J28" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K28" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L28" s="514" t="inlineStr"/>
+      <c r="M28" s="488" t="inlineStr">
         <is>
           <t>Saturated red-orange; active fire, heat</t>
         </is>
@@ -6408,8 +6669,17 @@
           <t>#FFAA00</t>
         </is>
       </c>
-      <c r="I29" s="515" t="inlineStr"/>
-      <c r="J29" s="488" t="inlineStr">
+      <c r="I29" s="484" t="n">
+        <v>40</v>
+      </c>
+      <c r="J29" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K29" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L29" s="515" t="inlineStr"/>
+      <c r="M29" s="488" t="inlineStr">
         <is>
           <t>Saturated pure orange; traffic, warnings</t>
         </is>
@@ -6444,8 +6714,17 @@
           <t>#FFFF00</t>
         </is>
       </c>
-      <c r="I30" s="516" t="inlineStr"/>
-      <c r="J30" s="488" t="inlineStr">
+      <c r="I30" s="484" t="n">
+        <v>60</v>
+      </c>
+      <c r="J30" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K30" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L30" s="516" t="inlineStr"/>
+      <c r="M30" s="488" t="inlineStr">
         <is>
           <t>Pure saturated yellow; maximum visibility</t>
         </is>
@@ -6480,8 +6759,17 @@
           <t>#AAFF00</t>
         </is>
       </c>
-      <c r="I31" s="517" t="inlineStr"/>
-      <c r="J31" s="488" t="inlineStr">
+      <c r="I31" s="484" t="n">
+        <v>80</v>
+      </c>
+      <c r="J31" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K31" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L31" s="517" t="inlineStr"/>
+      <c r="M31" s="488" t="inlineStr">
         <is>
           <t>Saturated lime; vivid vegetation markers</t>
         </is>
@@ -6516,8 +6804,17 @@
           <t>#55FF00</t>
         </is>
       </c>
-      <c r="I32" s="518" t="inlineStr"/>
-      <c r="J32" s="488" t="inlineStr">
+      <c r="I32" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="J32" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K32" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L32" s="518" t="inlineStr"/>
+      <c r="M32" s="488" t="inlineStr">
         <is>
           <t>Saturated grass green; bright greenspace</t>
         </is>
@@ -6552,8 +6849,17 @@
           <t>#00FFC5</t>
         </is>
       </c>
-      <c r="I33" s="519" t="inlineStr"/>
-      <c r="J33" s="488" t="inlineStr">
+      <c r="I33" s="484" t="n">
+        <v>166.4</v>
+      </c>
+      <c r="J33" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K33" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L33" s="519" t="inlineStr"/>
+      <c r="M33" s="488" t="inlineStr">
         <is>
           <t>Saturated cool seafoam; Caribbean water</t>
         </is>
@@ -6588,8 +6894,17 @@
           <t>#00C5FF</t>
         </is>
       </c>
-      <c r="I34" s="520" t="inlineStr"/>
-      <c r="J34" s="488" t="inlineStr">
+      <c r="I34" s="484" t="n">
+        <v>193.6</v>
+      </c>
+      <c r="J34" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K34" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L34" s="520" t="inlineStr"/>
+      <c r="M34" s="488" t="inlineStr">
         <is>
           <t>Saturated cool cyan; clear water bodies</t>
         </is>
@@ -6624,8 +6939,17 @@
           <t>#0082FF</t>
         </is>
       </c>
-      <c r="I35" s="521" t="inlineStr"/>
-      <c r="J35" s="488" t="inlineStr">
+      <c r="I35" s="484" t="n">
+        <v>209.4</v>
+      </c>
+      <c r="J35" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K35" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L35" s="521" t="inlineStr"/>
+      <c r="M35" s="488" t="inlineStr">
         <is>
           <t>Saturated cool azure; deeper water</t>
         </is>
@@ -6660,8 +6984,17 @@
           <t>#C500FF</t>
         </is>
       </c>
-      <c r="I36" s="522" t="inlineStr"/>
-      <c r="J36" s="488" t="inlineStr">
+      <c r="I36" s="484" t="n">
+        <v>286.4</v>
+      </c>
+      <c r="J36" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K36" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L36" s="522" t="inlineStr"/>
+      <c r="M36" s="488" t="inlineStr">
         <is>
           <t>Saturated cool violet; special features</t>
         </is>
@@ -6696,8 +7029,17 @@
           <t>#FF00C5</t>
         </is>
       </c>
-      <c r="I37" s="523" t="inlineStr"/>
-      <c r="J37" s="488" t="inlineStr">
+      <c r="I37" s="484" t="n">
+        <v>313.6</v>
+      </c>
+      <c r="J37" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K37" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="L37" s="523" t="inlineStr"/>
+      <c r="M37" s="488" t="inlineStr">
         <is>
           <t>Saturated warm hot pink; high-contrast markers</t>
         </is>
@@ -6732,8 +7074,17 @@
           <t>#B2B2B2</t>
         </is>
       </c>
-      <c r="I38" s="524" t="inlineStr"/>
-      <c r="J38" s="488" t="inlineStr">
+      <c r="I38" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" s="484" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="L38" s="524" t="inlineStr"/>
+      <c r="M38" s="488" t="inlineStr">
         <is>
           <t>Medium-light neutral; secondary fills</t>
         </is>
@@ -6768,8 +7119,17 @@
           <t>#E60000</t>
         </is>
       </c>
-      <c r="I39" s="525" t="inlineStr"/>
-      <c r="J39" s="488" t="inlineStr">
+      <c r="I39" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K39" s="484" t="n">
+        <v>90.2</v>
+      </c>
+      <c r="L39" s="525" t="inlineStr"/>
+      <c r="M39" s="488" t="inlineStr">
         <is>
           <t>Deep warm red; strong boundary lines</t>
         </is>
@@ -6804,8 +7164,17 @@
           <t>#E64C00</t>
         </is>
       </c>
-      <c r="I40" s="526" t="inlineStr"/>
-      <c r="J40" s="488" t="inlineStr">
+      <c r="I40" s="484" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="J40" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K40" s="484" t="n">
+        <v>90.2</v>
+      </c>
+      <c r="L40" s="526" t="inlineStr"/>
+      <c r="M40" s="488" t="inlineStr">
         <is>
           <t>Deep warm red-orange; active hazards</t>
         </is>
@@ -6840,8 +7209,17 @@
           <t>#E69800</t>
         </is>
       </c>
-      <c r="I41" s="527" t="inlineStr"/>
-      <c r="J41" s="488" t="inlineStr">
+      <c r="I41" s="484" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="J41" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K41" s="484" t="n">
+        <v>90.2</v>
+      </c>
+      <c r="L41" s="527" t="inlineStr"/>
+      <c r="M41" s="488" t="inlineStr">
         <is>
           <t>Rich warm orange; transit corridors</t>
         </is>
@@ -6876,8 +7254,17 @@
           <t>#E6E600</t>
         </is>
       </c>
-      <c r="I42" s="528" t="inlineStr"/>
-      <c r="J42" s="488" t="inlineStr">
+      <c r="I42" s="484" t="n">
+        <v>60</v>
+      </c>
+      <c r="J42" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K42" s="484" t="n">
+        <v>90.2</v>
+      </c>
+      <c r="L42" s="528" t="inlineStr"/>
+      <c r="M42" s="488" t="inlineStr">
         <is>
           <t>Rich warm lemon; highway markings</t>
         </is>
@@ -6912,8 +7299,17 @@
           <t>#98E600</t>
         </is>
       </c>
-      <c r="I43" s="529" t="inlineStr"/>
-      <c r="J43" s="488" t="inlineStr">
+      <c r="I43" s="484" t="n">
+        <v>80.3</v>
+      </c>
+      <c r="J43" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K43" s="484" t="n">
+        <v>90.2</v>
+      </c>
+      <c r="L43" s="529" t="inlineStr"/>
+      <c r="M43" s="488" t="inlineStr">
         <is>
           <t>Rich yellow-green; cropland, agriculture</t>
         </is>
@@ -6948,8 +7344,17 @@
           <t>#4CE600</t>
         </is>
       </c>
-      <c r="I44" s="530" t="inlineStr"/>
-      <c r="J44" s="488" t="inlineStr">
+      <c r="I44" s="484" t="n">
+        <v>100.2</v>
+      </c>
+      <c r="J44" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K44" s="484" t="n">
+        <v>90.2</v>
+      </c>
+      <c r="L44" s="530" t="inlineStr"/>
+      <c r="M44" s="488" t="inlineStr">
         <is>
           <t>Rich grass green; parks, forests</t>
         </is>
@@ -6984,8 +7389,17 @@
           <t>#00E6A9</t>
         </is>
       </c>
-      <c r="I45" s="531" t="inlineStr"/>
-      <c r="J45" s="488" t="inlineStr">
+      <c r="I45" s="484" t="n">
+        <v>164.1</v>
+      </c>
+      <c r="J45" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K45" s="484" t="n">
+        <v>90.2</v>
+      </c>
+      <c r="L45" s="531" t="inlineStr"/>
+      <c r="M45" s="488" t="inlineStr">
         <is>
           <t>Rich cool teal; estuaries, coastal zones</t>
         </is>
@@ -7020,8 +7434,17 @@
           <t>#00A9E6</t>
         </is>
       </c>
-      <c r="I46" s="532" t="inlineStr"/>
-      <c r="J46" s="488" t="inlineStr">
+      <c r="I46" s="484" t="n">
+        <v>195.9</v>
+      </c>
+      <c r="J46" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K46" s="484" t="n">
+        <v>90.2</v>
+      </c>
+      <c r="L46" s="532" t="inlineStr"/>
+      <c r="M46" s="488" t="inlineStr">
         <is>
           <t>Rich cool lagoon blue; lakes, bays</t>
         </is>
@@ -7056,8 +7479,17 @@
           <t>#005CE6</t>
         </is>
       </c>
-      <c r="I47" s="533" t="inlineStr"/>
-      <c r="J47" s="488" t="inlineStr">
+      <c r="I47" s="484" t="n">
+        <v>216</v>
+      </c>
+      <c r="J47" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K47" s="484" t="n">
+        <v>90.2</v>
+      </c>
+      <c r="L47" s="533" t="inlineStr"/>
+      <c r="M47" s="488" t="inlineStr">
         <is>
           <t>Rich cool deep blue; major waterways</t>
         </is>
@@ -7092,8 +7524,17 @@
           <t>#A900E6</t>
         </is>
       </c>
-      <c r="I48" s="534" t="inlineStr"/>
-      <c r="J48" s="488" t="inlineStr">
+      <c r="I48" s="484" t="n">
+        <v>284.1</v>
+      </c>
+      <c r="J48" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K48" s="484" t="n">
+        <v>90.2</v>
+      </c>
+      <c r="L48" s="534" t="inlineStr"/>
+      <c r="M48" s="488" t="inlineStr">
         <is>
           <t>Rich cool violet; zoning, boundaries</t>
         </is>
@@ -7128,8 +7569,17 @@
           <t>#E600A9</t>
         </is>
       </c>
-      <c r="I49" s="535" t="inlineStr"/>
-      <c r="J49" s="488" t="inlineStr">
+      <c r="I49" s="484" t="n">
+        <v>315.9</v>
+      </c>
+      <c r="J49" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K49" s="484" t="n">
+        <v>90.2</v>
+      </c>
+      <c r="L49" s="535" t="inlineStr"/>
+      <c r="M49" s="488" t="inlineStr">
         <is>
           <t>Rich warm magenta; distinctive features</t>
         </is>
@@ -7164,8 +7614,17 @@
           <t>#9C9C9C</t>
         </is>
       </c>
-      <c r="I50" s="536" t="inlineStr"/>
-      <c r="J50" s="488" t="inlineStr">
+      <c r="I50" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" s="484" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="L50" s="536" t="inlineStr"/>
+      <c r="M50" s="488" t="inlineStr">
         <is>
           <t>Medium neutral; base infrastructure</t>
         </is>
@@ -7200,8 +7659,17 @@
           <t>#A80000</t>
         </is>
       </c>
-      <c r="I51" s="537" t="inlineStr"/>
-      <c r="J51" s="488" t="inlineStr">
+      <c r="I51" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K51" s="484" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="L51" s="537" t="inlineStr"/>
+      <c r="M51" s="488" t="inlineStr">
         <is>
           <t>Deep warm brick; rail, transportation</t>
         </is>
@@ -7236,8 +7704,17 @@
           <t>#A83800</t>
         </is>
       </c>
-      <c r="I52" s="538" t="inlineStr"/>
-      <c r="J52" s="488" t="inlineStr">
+      <c r="I52" s="484" t="n">
+        <v>20</v>
+      </c>
+      <c r="J52" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K52" s="484" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="L52" s="538" t="inlineStr"/>
+      <c r="M52" s="488" t="inlineStr">
         <is>
           <t>Deep warm brown-red; industrial zones</t>
         </is>
@@ -7272,8 +7749,17 @@
           <t>#A87000</t>
         </is>
       </c>
-      <c r="I53" s="539" t="inlineStr"/>
-      <c r="J53" s="488" t="inlineStr">
+      <c r="I53" s="484" t="n">
+        <v>40</v>
+      </c>
+      <c r="J53" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K53" s="484" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="L53" s="539" t="inlineStr"/>
+      <c r="M53" s="488" t="inlineStr">
         <is>
           <t>Earthy warm caramel; soil, geology</t>
         </is>
@@ -7308,8 +7794,17 @@
           <t>#A8A800</t>
         </is>
       </c>
-      <c r="I54" s="540" t="inlineStr"/>
-      <c r="J54" s="488" t="inlineStr">
+      <c r="I54" s="484" t="n">
+        <v>60</v>
+      </c>
+      <c r="J54" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K54" s="484" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="L54" s="540" t="inlineStr"/>
+      <c r="M54" s="488" t="inlineStr">
         <is>
           <t>Earthy muted olive; scrubland, rangeland</t>
         </is>
@@ -7344,8 +7839,17 @@
           <t>#70A800</t>
         </is>
       </c>
-      <c r="I55" s="541" t="inlineStr"/>
-      <c r="J55" s="488" t="inlineStr">
+      <c r="I55" s="484" t="n">
+        <v>80</v>
+      </c>
+      <c r="J55" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K55" s="484" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="L55" s="541" t="inlineStr"/>
+      <c r="M55" s="488" t="inlineStr">
         <is>
           <t>Earthy cool olive; managed forest</t>
         </is>
@@ -7380,8 +7884,17 @@
           <t>#38A800</t>
         </is>
       </c>
-      <c r="I56" s="542" t="inlineStr"/>
-      <c r="J56" s="488" t="inlineStr">
+      <c r="I56" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="J56" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K56" s="484" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="L56" s="542" t="inlineStr"/>
+      <c r="M56" s="488" t="inlineStr">
         <is>
           <t>Deep cool forest-leaf; woodland areas</t>
         </is>
@@ -7416,8 +7929,17 @@
           <t>#00A884</t>
         </is>
       </c>
-      <c r="I57" s="543" t="inlineStr"/>
-      <c r="J57" s="488" t="inlineStr">
+      <c r="I57" s="484" t="n">
+        <v>167.1</v>
+      </c>
+      <c r="J57" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K57" s="484" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="L57" s="543" t="inlineStr"/>
+      <c r="M57" s="488" t="inlineStr">
         <is>
           <t>Deep cool teal-green; wetlands, marshes</t>
         </is>
@@ -7452,8 +7974,17 @@
           <t>#0084A8</t>
         </is>
       </c>
-      <c r="I58" s="544" t="inlineStr"/>
-      <c r="J58" s="488" t="inlineStr">
+      <c r="I58" s="484" t="n">
+        <v>192.9</v>
+      </c>
+      <c r="J58" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K58" s="484" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="L58" s="544" t="inlineStr"/>
+      <c r="M58" s="488" t="inlineStr">
         <is>
           <t>Deep cool teal-blue; deep lakes</t>
         </is>
@@ -7488,8 +8019,17 @@
           <t>#004DA8</t>
         </is>
       </c>
-      <c r="I59" s="545" t="inlineStr"/>
-      <c r="J59" s="488" t="inlineStr">
+      <c r="I59" s="484" t="n">
+        <v>212.5</v>
+      </c>
+      <c r="J59" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K59" s="484" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="L59" s="545" t="inlineStr"/>
+      <c r="M59" s="488" t="inlineStr">
         <is>
           <t>Deep cool denim blue; ocean, deep water</t>
         </is>
@@ -7524,8 +8064,17 @@
           <t>#8400A8</t>
         </is>
       </c>
-      <c r="I60" s="546" t="inlineStr"/>
-      <c r="J60" s="488" t="inlineStr">
+      <c r="I60" s="484" t="n">
+        <v>287.1</v>
+      </c>
+      <c r="J60" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K60" s="484" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="L60" s="546" t="inlineStr"/>
+      <c r="M60" s="488" t="inlineStr">
         <is>
           <t>Deep cool purple; political boundaries</t>
         </is>
@@ -7560,8 +8109,17 @@
           <t>#A80084</t>
         </is>
       </c>
-      <c r="I61" s="547" t="inlineStr"/>
-      <c r="J61" s="488" t="inlineStr">
+      <c r="I61" s="484" t="n">
+        <v>312.9</v>
+      </c>
+      <c r="J61" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K61" s="484" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="L61" s="547" t="inlineStr"/>
+      <c r="M61" s="488" t="inlineStr">
         <is>
           <t>Deep warm magenta; special overlays</t>
         </is>
@@ -7596,8 +8154,17 @@
           <t>#828282</t>
         </is>
       </c>
-      <c r="I62" s="548" t="inlineStr"/>
-      <c r="J62" s="488" t="inlineStr">
+      <c r="I62" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="K62" s="484" t="n">
+        <v>51</v>
+      </c>
+      <c r="L62" s="548" t="inlineStr"/>
+      <c r="M62" s="488" t="inlineStr">
         <is>
           <t>True middle gray; pavement, roads</t>
         </is>
@@ -7632,8 +8199,17 @@
           <t>#730000</t>
         </is>
       </c>
-      <c r="I63" s="549" t="inlineStr"/>
-      <c r="J63" s="488" t="inlineStr">
+      <c r="I63" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K63" s="484" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="L63" s="549" t="inlineStr"/>
+      <c r="M63" s="488" t="inlineStr">
         <is>
           <t>Very dark warm maroon; strong borders</t>
         </is>
@@ -7668,8 +8244,17 @@
           <t>#732600</t>
         </is>
       </c>
-      <c r="I64" s="550" t="inlineStr"/>
-      <c r="J64" s="488" t="inlineStr">
+      <c r="I64" s="484" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="J64" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K64" s="484" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="L64" s="550" t="inlineStr"/>
+      <c r="M64" s="488" t="inlineStr">
         <is>
           <t>Very dark warm red-brown; rail lines</t>
         </is>
@@ -7704,8 +8289,17 @@
           <t>#734C00</t>
         </is>
       </c>
-      <c r="I65" s="551" t="inlineStr"/>
-      <c r="J65" s="488" t="inlineStr">
+      <c r="I65" s="484" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="J65" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K65" s="484" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="L65" s="551" t="inlineStr"/>
+      <c r="M65" s="488" t="inlineStr">
         <is>
           <t>Very dark warm coffee; deep soil, bedrock</t>
         </is>
@@ -7740,8 +8334,17 @@
           <t>#737300</t>
         </is>
       </c>
-      <c r="I66" s="552" t="inlineStr"/>
-      <c r="J66" s="488" t="inlineStr">
+      <c r="I66" s="484" t="n">
+        <v>60</v>
+      </c>
+      <c r="J66" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K66" s="484" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="L66" s="552" t="inlineStr"/>
+      <c r="M66" s="488" t="inlineStr">
         <is>
           <t>Very dark muted olive; dry scrubland</t>
         </is>
@@ -7776,8 +8379,17 @@
           <t>#4C7300</t>
         </is>
       </c>
-      <c r="I67" s="553" t="inlineStr"/>
-      <c r="J67" s="488" t="inlineStr">
+      <c r="I67" s="484" t="n">
+        <v>80.3</v>
+      </c>
+      <c r="J67" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K67" s="484" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="L67" s="553" t="inlineStr"/>
+      <c r="M67" s="488" t="inlineStr">
         <is>
           <t>Very dark cool pine; conifer forest</t>
         </is>
@@ -7812,8 +8424,17 @@
           <t>#267300</t>
         </is>
       </c>
-      <c r="I68" s="554" t="inlineStr"/>
-      <c r="J68" s="488" t="inlineStr">
+      <c r="I68" s="484" t="n">
+        <v>100.2</v>
+      </c>
+      <c r="J68" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K68" s="484" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="L68" s="554" t="inlineStr"/>
+      <c r="M68" s="488" t="inlineStr">
         <is>
           <t>Very dark cool forest; dense woodland</t>
         </is>
@@ -7848,8 +8469,17 @@
           <t>#00734C</t>
         </is>
       </c>
-      <c r="I69" s="555" t="inlineStr"/>
-      <c r="J69" s="488" t="inlineStr">
+      <c r="I69" s="484" t="n">
+        <v>159.7</v>
+      </c>
+      <c r="J69" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K69" s="484" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="L69" s="555" t="inlineStr"/>
+      <c r="M69" s="488" t="inlineStr">
         <is>
           <t>Very dark cool teal; deep ocean water</t>
         </is>
@@ -7884,8 +8514,17 @@
           <t>#004C73</t>
         </is>
       </c>
-      <c r="I70" s="556" t="inlineStr"/>
-      <c r="J70" s="488" t="inlineStr">
+      <c r="I70" s="484" t="n">
+        <v>200.3</v>
+      </c>
+      <c r="J70" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K70" s="484" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="L70" s="556" t="inlineStr"/>
+      <c r="M70" s="488" t="inlineStr">
         <is>
           <t>Very dark cool blue; stormy seas</t>
         </is>
@@ -7920,8 +8559,17 @@
           <t>#002673</t>
         </is>
       </c>
-      <c r="I71" s="557" t="inlineStr"/>
-      <c r="J71" s="488" t="inlineStr">
+      <c r="I71" s="484" t="n">
+        <v>220.2</v>
+      </c>
+      <c r="J71" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K71" s="484" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="L71" s="557" t="inlineStr"/>
+      <c r="M71" s="488" t="inlineStr">
         <is>
           <t>Very dark cool navy; deep ocean, night</t>
         </is>
@@ -7956,8 +8604,17 @@
           <t>#4C0073</t>
         </is>
       </c>
-      <c r="I72" s="558" t="inlineStr"/>
-      <c r="J72" s="488" t="inlineStr">
+      <c r="I72" s="484" t="n">
+        <v>279.7</v>
+      </c>
+      <c r="J72" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K72" s="484" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="L72" s="558" t="inlineStr"/>
+      <c r="M72" s="488" t="inlineStr">
         <is>
           <t>Very dark cool purple-blue; specialty boundaries</t>
         </is>
@@ -7992,8 +8649,17 @@
           <t>#73004C</t>
         </is>
       </c>
-      <c r="I73" s="559" t="inlineStr"/>
-      <c r="J73" s="488" t="inlineStr">
+      <c r="I73" s="484" t="n">
+        <v>320.3</v>
+      </c>
+      <c r="J73" s="484" t="n">
+        <v>100</v>
+      </c>
+      <c r="K73" s="484" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="L73" s="559" t="inlineStr"/>
+      <c r="M73" s="488" t="inlineStr">
         <is>
           <t>Very dark balanced plum; distinctive districts</t>
         </is>
@@ -8028,8 +8694,17 @@
           <t>#686868</t>
         </is>
       </c>
-      <c r="I74" s="560" t="inlineStr"/>
-      <c r="J74" s="488" t="inlineStr">
+      <c r="I74" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="K74" s="484" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="L74" s="560" t="inlineStr"/>
+      <c r="M74" s="488" t="inlineStr">
         <is>
           <t>Medium-dark neutral; road networks</t>
         </is>
@@ -8064,8 +8739,17 @@
           <t>#D79E9E</t>
         </is>
       </c>
-      <c r="I75" s="561" t="inlineStr"/>
-      <c r="J75" s="488" t="inlineStr">
+      <c r="I75" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" s="484" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="K75" s="484" t="n">
+        <v>84.3</v>
+      </c>
+      <c r="L75" s="561" t="inlineStr"/>
+      <c r="M75" s="488" t="inlineStr">
         <is>
           <t>Muted warm dusty pink; faded residential</t>
         </is>
@@ -8100,8 +8784,17 @@
           <t>#D7B09E</t>
         </is>
       </c>
-      <c r="I76" s="562" t="inlineStr"/>
-      <c r="J76" s="488" t="inlineStr">
+      <c r="I76" s="484" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="J76" s="484" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="K76" s="484" t="n">
+        <v>84.3</v>
+      </c>
+      <c r="L76" s="562" t="inlineStr"/>
+      <c r="M76" s="488" t="inlineStr">
         <is>
           <t>Muted warm peach; weathered terracotta</t>
         </is>
@@ -8136,8 +8829,17 @@
           <t>#D7C29E</t>
         </is>
       </c>
-      <c r="I77" s="563" t="inlineStr"/>
-      <c r="J77" s="488" t="inlineStr">
+      <c r="I77" s="484" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="J77" s="484" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="K77" s="484" t="n">
+        <v>84.3</v>
+      </c>
+      <c r="L77" s="563" t="inlineStr"/>
+      <c r="M77" s="488" t="inlineStr">
         <is>
           <t>Muted warm beige; adobe, desert towns</t>
         </is>
@@ -8172,8 +8874,17 @@
           <t>#D7D79E</t>
         </is>
       </c>
-      <c r="I78" s="564" t="inlineStr"/>
-      <c r="J78" s="488" t="inlineStr">
+      <c r="I78" s="484" t="n">
+        <v>60</v>
+      </c>
+      <c r="J78" s="484" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="K78" s="484" t="n">
+        <v>84.3</v>
+      </c>
+      <c r="L78" s="564" t="inlineStr"/>
+      <c r="M78" s="488" t="inlineStr">
         <is>
           <t>Muted earthy pale yellow; dry grassland</t>
         </is>
@@ -8208,8 +8919,17 @@
           <t>#C7D79E</t>
         </is>
       </c>
-      <c r="I79" s="565" t="inlineStr"/>
-      <c r="J79" s="488" t="inlineStr">
+      <c r="I79" s="484" t="n">
+        <v>76.8</v>
+      </c>
+      <c r="J79" s="484" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="K79" s="484" t="n">
+        <v>84.3</v>
+      </c>
+      <c r="L79" s="565" t="inlineStr"/>
+      <c r="M79" s="488" t="inlineStr">
         <is>
           <t>Muted balanced pale green; sage scrubland</t>
         </is>
@@ -8244,8 +8964,17 @@
           <t>#B4D79E</t>
         </is>
       </c>
-      <c r="I80" s="566" t="inlineStr"/>
-      <c r="J80" s="488" t="inlineStr">
+      <c r="I80" s="484" t="n">
+        <v>96.8</v>
+      </c>
+      <c r="J80" s="484" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="K80" s="484" t="n">
+        <v>84.3</v>
+      </c>
+      <c r="L80" s="566" t="inlineStr"/>
+      <c r="M80" s="488" t="inlineStr">
         <is>
           <t>Muted cool dusty green; dried herbs, chaparral</t>
         </is>
@@ -8280,8 +9009,17 @@
           <t>#9ED7C2</t>
         </is>
       </c>
-      <c r="I81" s="567" t="inlineStr"/>
-      <c r="J81" s="488" t="inlineStr">
+      <c r="I81" s="484" t="n">
+        <v>157.9</v>
+      </c>
+      <c r="J81" s="484" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="K81" s="484" t="n">
+        <v>84.3</v>
+      </c>
+      <c r="L81" s="567" t="inlineStr"/>
+      <c r="M81" s="488" t="inlineStr">
         <is>
           <t>Muted cool pale teal; sea glass, estuary</t>
         </is>
@@ -8316,8 +9054,17 @@
           <t>#9EBBD7</t>
         </is>
       </c>
-      <c r="I82" s="568" t="inlineStr"/>
-      <c r="J82" s="488" t="inlineStr">
+      <c r="I82" s="484" t="n">
+        <v>209.5</v>
+      </c>
+      <c r="J82" s="484" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="K82" s="484" t="n">
+        <v>84.3</v>
+      </c>
+      <c r="L82" s="568" t="inlineStr"/>
+      <c r="M82" s="488" t="inlineStr">
         <is>
           <t>Muted cool dusty blue; distant mountains</t>
         </is>
@@ -8352,8 +9099,17 @@
           <t>#9EAAD7</t>
         </is>
       </c>
-      <c r="I83" s="569" t="inlineStr"/>
-      <c r="J83" s="488" t="inlineStr">
+      <c r="I83" s="484" t="n">
+        <v>227.4</v>
+      </c>
+      <c r="J83" s="484" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="K83" s="484" t="n">
+        <v>84.3</v>
+      </c>
+      <c r="L83" s="569" t="inlineStr"/>
+      <c r="M83" s="488" t="inlineStr">
         <is>
           <t>Muted cool periwinkle; faded denim, haze</t>
         </is>
@@ -8388,8 +9144,17 @@
           <t>#C29ED7</t>
         </is>
       </c>
-      <c r="I84" s="570" t="inlineStr"/>
-      <c r="J84" s="488" t="inlineStr">
+      <c r="I84" s="484" t="n">
+        <v>277.9</v>
+      </c>
+      <c r="J84" s="484" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="K84" s="484" t="n">
+        <v>84.3</v>
+      </c>
+      <c r="L84" s="570" t="inlineStr"/>
+      <c r="M84" s="488" t="inlineStr">
         <is>
           <t>Muted cool dusty lavender; dried flowers</t>
         </is>
@@ -8424,8 +9189,17 @@
           <t>#D69DBC</t>
         </is>
       </c>
-      <c r="I85" s="571" t="inlineStr"/>
-      <c r="J85" s="488" t="inlineStr">
+      <c r="I85" s="484" t="n">
+        <v>327.4</v>
+      </c>
+      <c r="J85" s="484" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="K85" s="484" t="n">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="L85" s="571" t="inlineStr"/>
+      <c r="M85" s="488" t="inlineStr">
         <is>
           <t>Muted warm dusty mauve; antique roses</t>
         </is>
@@ -8460,8 +9234,17 @@
           <t>#4E4E4E</t>
         </is>
       </c>
-      <c r="I86" s="572" t="inlineStr"/>
-      <c r="J86" s="488" t="inlineStr">
+      <c r="I86" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" s="484" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="L86" s="572" t="inlineStr"/>
+      <c r="M86" s="488" t="inlineStr">
         <is>
           <t>Dark neutral charcoal; major highways</t>
         </is>
@@ -8496,8 +9279,17 @@
           <t>#F57A7A</t>
         </is>
       </c>
-      <c r="I87" s="573" t="inlineStr"/>
-      <c r="J87" s="488" t="inlineStr">
+      <c r="I87" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J87" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K87" s="484" t="n">
+        <v>96.09999999999999</v>
+      </c>
+      <c r="L87" s="573" t="inlineStr"/>
+      <c r="M87" s="488" t="inlineStr">
         <is>
           <t>Medium warm coral-pink; salmon, residential</t>
         </is>
@@ -8532,8 +9324,17 @@
           <t>#F5A27A</t>
         </is>
       </c>
-      <c r="I88" s="574" t="inlineStr"/>
-      <c r="J88" s="488" t="inlineStr">
+      <c r="I88" s="484" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="J88" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K88" s="484" t="n">
+        <v>96.09999999999999</v>
+      </c>
+      <c r="L88" s="574" t="inlineStr"/>
+      <c r="M88" s="488" t="inlineStr">
         <is>
           <t>Medium warm peach; dusty sunset, suburbs</t>
         </is>
@@ -8568,8 +9369,17 @@
           <t>#F5CA7A</t>
         </is>
       </c>
-      <c r="I89" s="575" t="inlineStr"/>
-      <c r="J89" s="488" t="inlineStr">
+      <c r="I89" s="484" t="n">
+        <v>39</v>
+      </c>
+      <c r="J89" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K89" s="484" t="n">
+        <v>96.09999999999999</v>
+      </c>
+      <c r="L89" s="575" t="inlineStr"/>
+      <c r="M89" s="488" t="inlineStr">
         <is>
           <t>Medium warm tan; beach, sandy terrain</t>
         </is>
@@ -8604,8 +9414,17 @@
           <t>#F5F57A</t>
         </is>
       </c>
-      <c r="I90" s="576" t="inlineStr"/>
-      <c r="J90" s="488" t="inlineStr">
+      <c r="I90" s="484" t="n">
+        <v>60</v>
+      </c>
+      <c r="J90" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K90" s="484" t="n">
+        <v>96.09999999999999</v>
+      </c>
+      <c r="L90" s="576" t="inlineStr"/>
+      <c r="M90" s="488" t="inlineStr">
         <is>
           <t>Medium balanced yellow; soft cropland</t>
         </is>
@@ -8640,8 +9459,17 @@
           <t>#CDF57A</t>
         </is>
       </c>
-      <c r="I91" s="577" t="inlineStr"/>
-      <c r="J91" s="488" t="inlineStr">
+      <c r="I91" s="484" t="n">
+        <v>79.5</v>
+      </c>
+      <c r="J91" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K91" s="484" t="n">
+        <v>96.09999999999999</v>
+      </c>
+      <c r="L91" s="577" t="inlineStr"/>
+      <c r="M91" s="488" t="inlineStr">
         <is>
           <t>Medium balanced yellow-green; mixed vegetation</t>
         </is>
@@ -8676,8 +9504,17 @@
           <t>#A5F57A</t>
         </is>
       </c>
-      <c r="I92" s="578" t="inlineStr"/>
-      <c r="J92" s="488" t="inlineStr">
+      <c r="I92" s="484" t="n">
+        <v>99</v>
+      </c>
+      <c r="J92" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K92" s="484" t="n">
+        <v>96.09999999999999</v>
+      </c>
+      <c r="L92" s="578" t="inlineStr"/>
+      <c r="M92" s="488" t="inlineStr">
         <is>
           <t>Medium cool spring green; young crops</t>
         </is>
@@ -8712,8 +9549,17 @@
           <t>#7AF5CA</t>
         </is>
       </c>
-      <c r="I93" s="579" t="inlineStr"/>
-      <c r="J93" s="488" t="inlineStr">
+      <c r="I93" s="484" t="n">
+        <v>159</v>
+      </c>
+      <c r="J93" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K93" s="484" t="n">
+        <v>96.09999999999999</v>
+      </c>
+      <c r="L93" s="579" t="inlineStr"/>
+      <c r="M93" s="488" t="inlineStr">
         <is>
           <t>Medium cool mint; fresh water, streams</t>
         </is>
@@ -8748,8 +9594,17 @@
           <t>#7AB6F5</t>
         </is>
       </c>
-      <c r="I94" s="580" t="inlineStr"/>
-      <c r="J94" s="488" t="inlineStr">
+      <c r="I94" s="484" t="n">
+        <v>210.7</v>
+      </c>
+      <c r="J94" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K94" s="484" t="n">
+        <v>96.09999999999999</v>
+      </c>
+      <c r="L94" s="580" t="inlineStr"/>
+      <c r="M94" s="488" t="inlineStr">
         <is>
           <t>Medium cool sky blue; open water</t>
         </is>
@@ -8784,8 +9639,17 @@
           <t>#7A8EF5</t>
         </is>
       </c>
-      <c r="I95" s="581" t="inlineStr"/>
-      <c r="J95" s="488" t="inlineStr">
+      <c r="I95" s="484" t="n">
+        <v>230.2</v>
+      </c>
+      <c r="J95" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K95" s="484" t="n">
+        <v>96.09999999999999</v>
+      </c>
+      <c r="L95" s="581" t="inlineStr"/>
+      <c r="M95" s="488" t="inlineStr">
         <is>
           <t>Medium cool blue-violet; blueberry, dusk</t>
         </is>
@@ -8820,8 +9684,17 @@
           <t>#CA7AF5</t>
         </is>
       </c>
-      <c r="I96" s="582" t="inlineStr"/>
-      <c r="J96" s="488" t="inlineStr">
+      <c r="I96" s="484" t="n">
+        <v>279</v>
+      </c>
+      <c r="J96" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K96" s="484" t="n">
+        <v>96.09999999999999</v>
+      </c>
+      <c r="L96" s="582" t="inlineStr"/>
+      <c r="M96" s="488" t="inlineStr">
         <is>
           <t>Medium balanced orchid; zoning overlays</t>
         </is>
@@ -8856,8 +9729,17 @@
           <t>#F57AB6</t>
         </is>
       </c>
-      <c r="I97" s="583" t="inlineStr"/>
-      <c r="J97" s="488" t="inlineStr">
+      <c r="I97" s="484" t="n">
+        <v>330.7</v>
+      </c>
+      <c r="J97" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K97" s="484" t="n">
+        <v>96.09999999999999</v>
+      </c>
+      <c r="L97" s="583" t="inlineStr"/>
+      <c r="M97" s="488" t="inlineStr">
         <is>
           <t>Medium warm pink-magenta; notable boundaries</t>
         </is>
@@ -8892,8 +9774,17 @@
           <t>#343434</t>
         </is>
       </c>
-      <c r="I98" s="584" t="inlineStr"/>
-      <c r="J98" s="488" t="inlineStr">
+      <c r="I98" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J98" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="K98" s="484" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="L98" s="584" t="inlineStr"/>
+      <c r="M98" s="488" t="inlineStr">
         <is>
           <t>Very dark neutral; major rail, arterials</t>
         </is>
@@ -8928,8 +9819,17 @@
           <t>#CD6666</t>
         </is>
       </c>
-      <c r="I99" s="585" t="inlineStr"/>
-      <c r="J99" s="488" t="inlineStr">
+      <c r="I99" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J99" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K99" s="484" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="L99" s="585" t="inlineStr"/>
+      <c r="M99" s="488" t="inlineStr">
         <is>
           <t>Muted warm brick pink; old rooftops</t>
         </is>
@@ -8964,8 +9864,17 @@
           <t>#CD8966</t>
         </is>
       </c>
-      <c r="I100" s="586" t="inlineStr"/>
-      <c r="J100" s="488" t="inlineStr">
+      <c r="I100" s="484" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="J100" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K100" s="484" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="L100" s="586" t="inlineStr"/>
+      <c r="M100" s="488" t="inlineStr">
         <is>
           <t>Muted warm tan; suede, leather earthtones</t>
         </is>
@@ -9000,8 +9909,17 @@
           <t>#CDAA66</t>
         </is>
       </c>
-      <c r="I101" s="587" t="inlineStr"/>
-      <c r="J101" s="488" t="inlineStr">
+      <c r="I101" s="484" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="J101" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K101" s="484" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="L101" s="587" t="inlineStr"/>
+      <c r="M101" s="488" t="inlineStr">
         <is>
           <t>Muted warm ochre; clay pottery, pueblo</t>
         </is>
@@ -9036,8 +9954,17 @@
           <t>#CDCD66</t>
         </is>
       </c>
-      <c r="I102" s="588" t="inlineStr"/>
-      <c r="J102" s="488" t="inlineStr">
+      <c r="I102" s="484" t="n">
+        <v>60</v>
+      </c>
+      <c r="J102" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K102" s="484" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="L102" s="588" t="inlineStr"/>
+      <c r="M102" s="488" t="inlineStr">
         <is>
           <t>Muted balanced yellow-olive; dried herbs</t>
         </is>
@@ -9072,8 +9999,17 @@
           <t>#ABCD66</t>
         </is>
       </c>
-      <c r="I103" s="589" t="inlineStr"/>
-      <c r="J103" s="488" t="inlineStr">
+      <c r="I103" s="484" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="J103" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K103" s="484" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="L103" s="589" t="inlineStr"/>
+      <c r="M103" s="488" t="inlineStr">
         <is>
           <t>Muted cool olive-green; pasture, rangeland</t>
         </is>
@@ -9108,8 +10044,17 @@
           <t>#89CD66</t>
         </is>
       </c>
-      <c r="I104" s="590" t="inlineStr"/>
-      <c r="J104" s="488" t="inlineStr">
+      <c r="I104" s="484" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="J104" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K104" s="484" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="L104" s="590" t="inlineStr"/>
+      <c r="M104" s="488" t="inlineStr">
         <is>
           <t>Muted cool leaf green; shaded ferns, understory</t>
         </is>
@@ -9144,8 +10089,17 @@
           <t>#66CDAB</t>
         </is>
       </c>
-      <c r="I105" s="591" t="inlineStr"/>
-      <c r="J105" s="488" t="inlineStr">
+      <c r="I105" s="484" t="n">
+        <v>160.2</v>
+      </c>
+      <c r="J105" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K105" s="484" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="L105" s="591" t="inlineStr"/>
+      <c r="M105" s="488" t="inlineStr">
         <is>
           <t>Muted cool jade; stream beds, wetlands</t>
         </is>
@@ -9180,8 +10134,17 @@
           <t>#6699CD</t>
         </is>
       </c>
-      <c r="I106" s="592" t="inlineStr"/>
-      <c r="J106" s="488" t="inlineStr">
+      <c r="I106" s="484" t="n">
+        <v>210.3</v>
+      </c>
+      <c r="J106" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K106" s="484" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="L106" s="592" t="inlineStr"/>
+      <c r="M106" s="488" t="inlineStr">
         <is>
           <t>Muted cool ocean blue; coastal waters</t>
         </is>
@@ -9216,8 +10179,17 @@
           <t>#6677CD</t>
         </is>
       </c>
-      <c r="I107" s="593" t="inlineStr"/>
-      <c r="J107" s="488" t="inlineStr">
+      <c r="I107" s="484" t="n">
+        <v>230.1</v>
+      </c>
+      <c r="J107" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K107" s="484" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="L107" s="593" t="inlineStr"/>
+      <c r="M107" s="488" t="inlineStr">
         <is>
           <t>Muted cool slate; twilight sky, deep lakes</t>
         </is>
@@ -9252,8 +10224,17 @@
           <t>#AA66CD</t>
         </is>
       </c>
-      <c r="I108" s="594" t="inlineStr"/>
-      <c r="J108" s="488" t="inlineStr">
+      <c r="I108" s="484" t="n">
+        <v>279.6</v>
+      </c>
+      <c r="J108" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K108" s="484" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="L108" s="594" t="inlineStr"/>
+      <c r="M108" s="488" t="inlineStr">
         <is>
           <t>Muted cool violet; aster flower, overlays</t>
         </is>
@@ -9288,8 +10269,17 @@
           <t>#CD6699</t>
         </is>
       </c>
-      <c r="I109" s="595" t="inlineStr"/>
-      <c r="J109" s="488" t="inlineStr">
+      <c r="I109" s="484" t="n">
+        <v>330.3</v>
+      </c>
+      <c r="J109" s="484" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K109" s="484" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="L109" s="595" t="inlineStr"/>
+      <c r="M109" s="488" t="inlineStr">
         <is>
           <t>Muted balanced rose; flower gardens, accents</t>
         </is>
@@ -9324,8 +10314,17 @@
           <t>#000000</t>
         </is>
       </c>
-      <c r="I110" s="596" t="inlineStr"/>
-      <c r="J110" s="488" t="inlineStr">
+      <c r="I110" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J110" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="K110" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="L110" s="596" t="inlineStr"/>
+      <c r="M110" s="488" t="inlineStr">
         <is>
           <t>Pure black; outlines, text, maximum contrast</t>
         </is>
@@ -9360,8 +10359,17 @@
           <t>#894444</t>
         </is>
       </c>
-      <c r="I111" s="597" t="inlineStr"/>
-      <c r="J111" s="488" t="inlineStr">
+      <c r="I111" s="484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J111" s="484" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="K111" s="484" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="L111" s="597" t="inlineStr"/>
+      <c r="M111" s="488" t="inlineStr">
         <is>
           <t>Very dark warm burgundy; old leather, railroads</t>
         </is>
@@ -9396,8 +10404,17 @@
           <t>#895A44</t>
         </is>
       </c>
-      <c r="I112" s="598" t="inlineStr"/>
-      <c r="J112" s="488" t="inlineStr">
+      <c r="I112" s="484" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="J112" s="484" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="K112" s="484" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="L112" s="598" t="inlineStr"/>
+      <c r="M112" s="488" t="inlineStr">
         <is>
           <t>Very dark warm chocolate; deep soil, tracks</t>
         </is>
@@ -9432,8 +10449,17 @@
           <t>#897044</t>
         </is>
       </c>
-      <c r="I113" s="599" t="inlineStr"/>
-      <c r="J113" s="488" t="inlineStr">
+      <c r="I113" s="484" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="J113" s="484" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="K113" s="484" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="L113" s="599" t="inlineStr"/>
+      <c r="M113" s="488" t="inlineStr">
         <is>
           <t>Very dark warm earth; aged saddle, bedrock</t>
         </is>
@@ -9468,8 +10494,17 @@
           <t>#898944</t>
         </is>
       </c>
-      <c r="I114" s="600" t="inlineStr"/>
-      <c r="J114" s="488" t="inlineStr">
+      <c r="I114" s="484" t="n">
+        <v>60</v>
+      </c>
+      <c r="J114" s="484" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="K114" s="484" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="L114" s="600" t="inlineStr"/>
+      <c r="M114" s="488" t="inlineStr">
         <is>
           <t>Very dark earthy olive; lichen, weathered stone</t>
         </is>
@@ -9504,8 +10539,17 @@
           <t>#728944</t>
         </is>
       </c>
-      <c r="I115" s="601" t="inlineStr"/>
-      <c r="J115" s="488" t="inlineStr">
+      <c r="I115" s="484" t="n">
+        <v>80</v>
+      </c>
+      <c r="J115" s="484" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="K115" s="484" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="L115" s="601" t="inlineStr"/>
+      <c r="M115" s="488" t="inlineStr">
         <is>
           <t>Very dark earthy olive-green; forest moss</t>
         </is>
@@ -9540,8 +10584,17 @@
           <t>#5C8944</t>
         </is>
       </c>
-      <c r="I116" s="602" t="inlineStr"/>
-      <c r="J116" s="488" t="inlineStr">
+      <c r="I116" s="484" t="n">
+        <v>99.09999999999999</v>
+      </c>
+      <c r="J116" s="484" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="K116" s="484" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="L116" s="602" t="inlineStr"/>
+      <c r="M116" s="488" t="inlineStr">
         <is>
           <t>Very dark cool green; pond algae, bog</t>
         </is>
@@ -9576,8 +10629,17 @@
           <t>#448970</t>
         </is>
       </c>
-      <c r="I117" s="603" t="inlineStr"/>
-      <c r="J117" s="488" t="inlineStr">
+      <c r="I117" s="484" t="n">
+        <v>158.3</v>
+      </c>
+      <c r="J117" s="484" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="K117" s="484" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="L117" s="603" t="inlineStr"/>
+      <c r="M117" s="488" t="inlineStr">
         <is>
           <t>Very dark cool teal-green; deep forest shade</t>
         </is>
@@ -9612,8 +10674,17 @@
           <t>#446589</t>
         </is>
       </c>
-      <c r="I118" s="604" t="inlineStr"/>
-      <c r="J118" s="488" t="inlineStr">
+      <c r="I118" s="484" t="n">
+        <v>211.3</v>
+      </c>
+      <c r="J118" s="484" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="K118" s="484" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="L118" s="604" t="inlineStr"/>
+      <c r="M118" s="488" t="inlineStr">
         <is>
           <t>Very dark cool muted blue; denim at dusk</t>
         </is>
@@ -9648,8 +10719,17 @@
           <t>#264F89</t>
         </is>
       </c>
-      <c r="I119" s="605" t="inlineStr"/>
-      <c r="J119" s="488" t="inlineStr">
+      <c r="I119" s="484" t="n">
+        <v>215.2</v>
+      </c>
+      <c r="J119" s="484" t="n">
+        <v>72.3</v>
+      </c>
+      <c r="K119" s="484" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="L119" s="605" t="inlineStr"/>
+      <c r="M119" s="488" t="inlineStr">
         <is>
           <t>Very dark cool navy; glacier ice, deep sea</t>
         </is>
@@ -9684,8 +10764,17 @@
           <t>#704489</t>
         </is>
       </c>
-      <c r="I120" s="606" t="inlineStr"/>
-      <c r="J120" s="488" t="inlineStr">
+      <c r="I120" s="484" t="n">
+        <v>278.3</v>
+      </c>
+      <c r="J120" s="484" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="K120" s="484" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="L120" s="606" t="inlineStr"/>
+      <c r="M120" s="488" t="inlineStr">
         <is>
           <t>Very dark cool purple; the berry itself</t>
         </is>
@@ -9720,15 +10809,24 @@
           <t>#894465</t>
         </is>
       </c>
-      <c r="I121" s="607" t="inlineStr"/>
-      <c r="J121" s="488" t="inlineStr">
+      <c r="I121" s="484" t="n">
+        <v>331.3</v>
+      </c>
+      <c r="J121" s="484" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="K121" s="484" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="L121" s="607" t="inlineStr"/>
+      <c r="M121" s="488" t="inlineStr">
         <is>
           <t>Very dark warm wine; wine in shadow</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J121"/>
+  <autoFilter ref="A1:M121"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Correct Glacier Blue source values and sync palette deliverables
</commit_message>
<xml_diff>
--- a/color-palettes/arcmap-standard-palette/ArcMap_Color_Palette.xlsx
+++ b/color-palettes/arcmap-standard-palette/ArcMap_Color_Palette.xlsx
@@ -813,8 +813,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00264F89"/>
-        <bgColor rgb="00264F89"/>
+        <fgColor rgb="00444F89"/>
+        <bgColor rgb="00444F89"/>
       </patternFill>
     </fill>
     <fill>
@@ -5185,7 +5185,7 @@
       </c>
       <c r="J41" s="456" t="inlineStr">
         <is>
-          <t>38, 79, 137</t>
+          <t>68, 79, 137</t>
         </is>
       </c>
       <c r="K41" s="457" t="inlineStr">
@@ -5247,7 +5247,7 @@
       </c>
       <c r="J42" s="468" t="inlineStr">
         <is>
-          <t>#264F89</t>
+          <t>#444F89</t>
         </is>
       </c>
       <c r="K42" s="469" t="inlineStr">
@@ -10706,7 +10706,7 @@
         </is>
       </c>
       <c r="E119" s="484" t="n">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="F119" s="484" t="n">
         <v>79</v>
@@ -10716,14 +10716,14 @@
       </c>
       <c r="H119" s="486" t="inlineStr">
         <is>
-          <t>#264F89</t>
+          <t>#444F89</t>
         </is>
       </c>
       <c r="I119" s="484" t="n">
-        <v>215.2</v>
+        <v>230.4</v>
       </c>
       <c r="J119" s="484" t="n">
-        <v>72.3</v>
+        <v>50.4</v>
       </c>
       <c r="K119" s="484" t="n">
         <v>53.7</v>

</xml_diff>